<commit_message>
style: chuẩn hóa biểu mẫu BM - dấu chấm điền tay, giãn dòng Word, gọn header Excel
- Word: placeholder gạch dưới -> dấu chấm; giãn dòng 1.5 cho đoạn thân (trừ trong bảng)
- Excel: placeholder -> dấu chấm ở trường thông tin; bỏ cột trống dư cuối
- Excel: gộp ô khối mã số/ngày/lần ban hành vừa đủ, ưu tiên bề rộng tên công ty
- Thêm scripts/refine_bm_forms.py để tái áp dụng chỉnh sửa hàng loạt
</commit_message>
<xml_diff>
--- a/bm/KD/ISO.BM-KD-02-01 Bảng báo giá.xlsx
+++ b/bm/KD/ISO.BM-KD-02-01 Bảng báo giá.xlsx
@@ -63,7 +63,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -85,11 +85,110 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -120,6 +219,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -486,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -500,50 +611,50 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>CÔNG TY QS TECHNOLOGY</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="B1" s="13" t="n"/>
+      <c r="C1" s="13" t="n"/>
+      <c r="D1" s="13" t="n"/>
+      <c r="E1" s="13" t="n"/>
+      <c r="F1" s="13" t="n"/>
+      <c r="G1" s="14" t="inlineStr">
         <is>
           <t>Mã số: ISO.BM-KD-02-01</t>
         </is>
       </c>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="H1" s="13" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="A2" s="13" t="n"/>
+      <c r="B2" s="13" t="n"/>
+      <c r="C2" s="13" t="n"/>
+      <c r="D2" s="13" t="n"/>
+      <c r="E2" s="13" t="n"/>
+      <c r="F2" s="13" t="n"/>
+      <c r="G2" s="15" t="inlineStr">
         <is>
           <t>Ngày ban hành: 15/06/2026</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
+      <c r="H2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="A3" s="13" t="n"/>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="n"/>
+      <c r="F3" s="13" t="n"/>
+      <c r="G3" s="15" t="inlineStr">
         <is>
           <t>Lần ban hành: 01</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
+      <c r="H3" s="13" t="n"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -555,34 +666,34 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Kính gửi (Khách hàng):  ________________________________</t>
+          <t>Kính gửi (Khách hàng):  ................................</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Người liên hệ:  ________________________________</t>
+          <t>Người liên hệ:  ................................</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Điện thoại:  ________________________________</t>
+          <t>Điện thoại:  ................................</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Ngày báo giá:  ________________________________</t>
+          <t>Ngày báo giá:  ................................</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Số báo giá:  ________________________________</t>
+          <t>Số báo giá:  ................................</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Hiệu lực:  ________________________________</t>
+          <t>Hiệu lực:  ................................</t>
         </is>
       </c>
     </row>
@@ -714,6 +825,12 @@
           <t>Cộng tiền hàng:</t>
         </is>
       </c>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="16" t="n"/>
+      <c r="E16" s="16" t="n"/>
+      <c r="F16" s="16" t="n"/>
+      <c r="G16" s="17" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
@@ -721,6 +838,12 @@
           <t>Thuế VAT 10%:</t>
         </is>
       </c>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
+      <c r="E17" s="16" t="n"/>
+      <c r="F17" s="16" t="n"/>
+      <c r="G17" s="17" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -728,28 +851,34 @@
           <t>TỔNG CỘNG THANH TOÁN:</t>
         </is>
       </c>
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="16" t="n"/>
+      <c r="E18" s="16" t="n"/>
+      <c r="F18" s="16" t="n"/>
+      <c r="G18" s="17" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Bằng chữ: ___________________________________________________________</t>
+          <t>Bằng chữ: ...........................................................</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>Điều kiện thanh toán:  ________________________________</t>
+          <t>Điều kiện thanh toán:  ................................</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Thời gian giao hàng:  ________________________________</t>
+          <t>Thời gian giao hàng:  ................................</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>Bảo hành:  ________________________________</t>
+          <t>Bảo hành:  ................................</t>
         </is>
       </c>
     </row>
@@ -796,31 +925,31 @@
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="A17:G17"/>
+    <mergeCell ref="G2:H2"/>
     <mergeCell ref="A24:H24"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="E3:H3"/>
     <mergeCell ref="A25:H25"/>
-    <mergeCell ref="G20:I20"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="C22:D22"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="E5:H5"/>
+    <mergeCell ref="G3:H3"/>
     <mergeCell ref="A26:H26"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A1:D3"/>
     <mergeCell ref="A16:G16"/>
-    <mergeCell ref="E1:H1"/>
     <mergeCell ref="A23:B23"/>
     <mergeCell ref="D20:F20"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="A22:B22"/>
     <mergeCell ref="A4:H4"/>
+    <mergeCell ref="G20:H20"/>
     <mergeCell ref="A18:G18"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F3"/>
     <mergeCell ref="A19:H19"/>
     <mergeCell ref="E22:F22"/>
-    <mergeCell ref="E2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9"/>

</xml_diff>